<commit_message>
Add step-by-step usage and generation instructions
Expand the budget template's "How to use" tab and README with numbered,
step-by-step instructions covering both how to use the budget sheet
(Part A) and how to regenerate the workbook from the script (Part B).
Improve the How-to-use row-height heuristic so longer steps don't clip.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYLX9i8sJe3yBtAYwbeeq8
</commit_message>
<xml_diff>
--- a/budget-template/Hackathon_Innovation_Sprint_Budget_Template.xlsx
+++ b/budget-template/Hackathon_Innovation_Sprint_Budget_Template.xlsx
@@ -704,7 +704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B23"/>
+  <dimension ref="B2:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -728,7 +728,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="33" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Plan the cost of a 20-pax or 50-pax hackathon / innovation sprint, then track budget vs. actual spend on a live project — with automatic flags and a structured place to explain the big swings.</t>
@@ -745,28 +745,28 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="33" customHeight="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>1.  Budget vs Actual  —  the working sheet. Pick your event size, set budgets, log actuals. Any line item that runs &gt;20% over budget is flagged red and a reason becomes required.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="33" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>2.  Dashboard  —  auto-calculated roll-up by category, totals, and the list of flagged over-budget items. Nothing to fill in here.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="33" customHeight="1">
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t>3.  Impact &amp; Opportunities  —  log the spend that punched above its weight and the future opportunities it opened.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="33" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t>4.  Over-Budget Deep Dive  —  for each flagged item: the reason, the impact it actually delivered, and the way forward.</t>
@@ -779,71 +779,172 @@
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>HOW TO USE IT</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+          <t>PART A — STEP-BY-STEP: HOW TO USE THE BUDGET SHEET</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Step 1  —  On 'Budget vs Actual', fill the project header and choose Event size (20 or 50) from the dropdown. The Budgeted column auto-fills from the matching estimate; overwrite any cell with your real quote.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+          <t>Step 1  —  Open the 'Budget vs Actual' tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="33" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Step 2  —  As money is committed, enter the Actual for each line. Variance ($ and %) and the over-budget flag calculate automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+          <t>Step 2  —  Fill the header: Project / Client name, Event date, Currency (default SGD), Contingency % (default 10%), Variance threshold (default 20%) and Prepared by.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="33" customHeight="1">
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Step 3  —  Whenever 'Flag' shows ⚠ OVER, write the circumstance in the Reason column. This is the audit trail for spend that ran &gt;20% hot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>Step 3  —  Choose Event size (pax) from the dropdown — 20 or 50. The Budgeted column auto-fills from the matching estimate column for every line item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Step 4  —  After the event, complete 'Impact &amp; Opportunities' and 'Over-Budget Deep Dive' to close the loop on value and learnings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" t="inlineStr"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="2" t="inlineStr">
+          <t>Step 4  —  Replace the placeholder estimates with your real quotes. Edit the 'Est. 20 pax' / 'Est. 50 pax' cells (or type directly over the Budgeted cell) so the figures reflect your suppliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="33" customHeight="1">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Step 5  —  Add or remove line items to suit the event. Keep each row's Category text intact — the Dashboard rolls up by Category, so a blank/typo category drops the row from the totals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="33" customHeight="1">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Step 6  —  As costs are committed, enter each line's Actual (the grey cells). Variance ($), Variance % and the Flag calculate automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="33" customHeight="1">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Step 7  —  Watch the Flag column. ⚠ OVER (red) = more than +20% over budget; 'under' (green) = more than 20% under; 'ok' = within range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="33" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Step 8  —  For every ⚠ OVER line, write the circumstance in the Reason column. The cell stays amber until you do — this is your audit trail for big discrepancies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="33" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Step 9  —  Check the Dashboard tab for the category roll-up and headline KPIs (total budgeted, total actual, variance, and how many lines are flagged). It updates itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="33" customHeight="1">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Step 10  —  After the event, complete 'Impact &amp; Opportunities' (value created + doors opened) and 'Over-Budget Deep Dive' (reason → real impact → way forward) for each flagged item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>PART B — STEP-BY-STEP: HOW TO (RE)GENERATE THIS WORKBOOK</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="33" customHeight="1">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>The .xlsx is produced by a script, so you can regenerate it after changing line items, default amounts, currency, or branding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Step 1  —  Make sure Python 3 is installed:  python3 --version</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Step 2  —  Install the one dependency:  pip install openpyxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Step 3  —  Open generate_budget_template.py and edit the ITEMS list to change line items or placeholder estimates (each entry is: Category, Line item, Description, Est. 20 pax, Est. 50 pax). Header defaults (currency 'SGD', contingency 0.10, threshold 0.20) live in the 'hdr' dictionary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Step 4  —  From the budget-template folder, run:  python3 generate_budget_template.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="33" customHeight="1">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Step 5  —  The script overwrites Hackathon_Innovation_Sprint_Budget_Template.xlsx and prints a confirmation (line-item count + row range). Open the new file to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="33" customHeight="1">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Step 6  —  (Optional) To use it in Google Sheets: File → Import → Upload the .xlsx, then choose 'Replace spreadsheet'. Formulas, dropdowns and formatting carry over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>CONVENTIONS</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="B20" s="3" t="inlineStr">
+    <row r="35" ht="33" customHeight="1">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>•  Amounts shipped in the template are ILLUSTRATIVE planning placeholders — replace them with your own quotes.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="3" t="inlineStr">
+    <row r="36" ht="33" customHeight="1">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>•  Set your currency once in the header cell on 'Budget vs Actual'; it is shown on the Dashboard too.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="B22" s="3" t="inlineStr">
+    <row r="37" ht="33" customHeight="1">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>•  Items tagged '(good-to-have)' are optional client-rapport extras — keep, cut, or cost as the relationship warrants.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="3" t="inlineStr">
+    <row r="38" ht="33" customHeight="1">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>•  The +20% threshold is the trigger for an explanation. You can change it in the header (Variance threshold cell).</t>
         </is>

</xml_diff>

<commit_message>
Add steps for creating a new budget sheet per event
Add a "creating a new budget sheet for a new event" walkthrough (copy the
master, rename per engagement, clear actuals/reasons, set the header) to
both the workbook's How-to-use tab and the README, and renumber the
script regeneration steps to Part C.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYLX9i8sJe3yBtAYwbeeq8
</commit_message>
<xml_diff>
--- a/budget-template/Hackathon_Innovation_Sprint_Budget_Template.xlsx
+++ b/budget-template/Hackathon_Innovation_Sprint_Budget_Template.xlsx
@@ -704,7 +704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B38"/>
+  <dimension ref="B2:B49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -859,92 +859,165 @@
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>PART B — STEP-BY-STEP: HOW TO (RE)GENERATE THIS WORKBOOK</t>
+          <t>PART B — STEP-BY-STEP: CREATING A NEW BUDGET SHEET FOR A NEW EVENT</t>
         </is>
       </c>
     </row>
     <row r="26" ht="33" customHeight="1">
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>The .xlsx is produced by a script, so you can regenerate it after changing line items, default amounts, currency, or branding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
+          <t>Use one file per event and keep this template as a clean master — don't track a live project in the master copy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="33" customHeight="1">
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Step 1  —  Make sure Python 3 is installed:  python3 --version</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
+          <t>Step 1  —  Make a copy of the file. In Excel: File → Save As. In Google Sheets: File → Make a copy. (Or regenerate a fresh blank from the script — see Part C.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="33" customHeight="1">
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Step 2  —  Install the one dependency:  pip install openpyxl</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="48" customHeight="1">
+          <t>Step 2  —  Name the copy for the event, e.g. 2026-08_AcmeCorp_Sprint_Budget.xlsx, so each engagement has its own file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="33" customHeight="1">
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Step 3  —  Open generate_budget_template.py and edit the ITEMS list to change line items or placeholder estimates (each entry is: Category, Line item, Description, Est. 20 pax, Est. 50 pax). Header defaults (currency 'SGD', contingency 0.10, threshold 0.20) live in the 'hdr' dictionary.</t>
+          <t>Step 3  —  Open the copy's 'Budget vs Actual' tab and fill the header: Project / Client, Event date, Currency, Contingency %, Variance threshold, Prepared by.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Step 4  —  From the budget-template folder, run:  python3 generate_budget_template.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="33" customHeight="1">
+          <t>Step 4  —  Pick the Event size (20 or 50) from the dropdown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1">
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Step 5  —  The script overwrites Hackathon_Innovation_Sprint_Budget_Template.xlsx and prints a confirmation (line-item count + row range). Open the new file to verify.</t>
+          <t>Step 5  —  Clear any leftover entries so the sheet starts fresh — delete anything in the Actual and Reason columns (the master ships with these empty; this matters only if you copied a worked example).</t>
         </is>
       </c>
     </row>
     <row r="32" ht="33" customHeight="1">
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Step 6  —  (Optional) To use it in Google Sheets: File → Import → Upload the .xlsx, then choose 'Replace spreadsheet'. Formulas, dropdowns and formatting carry over.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" t="inlineStr"/>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>CONVENTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="33" customHeight="1">
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>•  Amounts shipped in the template are ILLUSTRATIVE planning placeholders — replace them with your own quotes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="33" customHeight="1">
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>•  Set your currency once in the header cell on 'Budget vs Actual'; it is shown on the Dashboard too.</t>
+          <t>Step 6  —  Replace the placeholder estimates with this event's quotes, and add/remove line items as needed (keep the Category text on every row).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="33" customHeight="1">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Step 7  —  Clear the 'Impact &amp; Opportunities' and 'Over-Budget Deep Dive' tabs of any prior entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Step 8  —  Save. Now follow Part A to run budget vs actual through the event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>PART C — STEP-BY-STEP: HOW TO (RE)GENERATE THIS WORKBOOK</t>
         </is>
       </c>
     </row>
     <row r="37" ht="33" customHeight="1">
       <c r="B37" s="3" t="inlineStr">
         <is>
+          <t>The .xlsx is produced by a script, so you can regenerate a fresh blank master after changing line items, default amounts, currency, or branding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Step 1  —  Make sure Python 3 is installed:  python3 --version</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Step 2  —  Install the one dependency:  pip install openpyxl</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Step 3  —  Open generate_budget_template.py and edit the ITEMS list to change line items or placeholder estimates (each entry is: Category, Line item, Description, Est. 20 pax, Est. 50 pax). Header defaults (currency 'SGD', contingency 0.10, threshold 0.20) live in the 'hdr' dictionary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Step 4  —  From the budget-template folder, run:  python3 generate_budget_template.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="33" customHeight="1">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Step 5  —  The script overwrites Hackathon_Innovation_Sprint_Budget_Template.xlsx and prints a confirmation (line-item count + row range). Open the new file to verify.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="33" customHeight="1">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Step 6  —  (Optional) To use it in Google Sheets: File → Import → Upload the .xlsx, then choose 'Replace spreadsheet'. Formulas, dropdowns and formatting carry over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>CONVENTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="33" customHeight="1">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>•  Amounts shipped in the template are ILLUSTRATIVE planning placeholders — replace them with your own quotes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="33" customHeight="1">
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>•  Set your currency once in the header cell on 'Budget vs Actual'; it is shown on the Dashboard too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="33" customHeight="1">
+      <c r="B48" s="3" t="inlineStr">
+        <is>
           <t>•  Items tagged '(good-to-have)' are optional client-rapport extras — keep, cut, or cost as the relationship warrants.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="33" customHeight="1">
-      <c r="B38" s="3" t="inlineStr">
+    <row r="49" ht="33" customHeight="1">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>•  The +20% threshold is the trigger for an explanation. You can change it in the header (Variance threshold cell).</t>
         </is>

</xml_diff>